<commit_message>
Update script scan price theo các version, script đoc concentrated pool thuận và đảo
</commit_message>
<xml_diff>
--- a/tests/datatest/ListPriceLeverage.xlsx
+++ b/tests/datatest/ListPriceLeverage.xlsx
@@ -9,13 +9,14 @@
   <sheets>
     <sheet name="List token" sheetId="1" r:id="rId1"/>
     <sheet name="Market info" sheetId="2" r:id="rId2"/>
+    <sheet name="Pool &amp; dToken" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="50">
   <si>
     <t>token</t>
   </si>
@@ -156,6 +157,15 @@
   </si>
   <si>
     <t>sADA</t>
+  </si>
+  <si>
+    <t>73f29518da0013a671458d52624a4828c5b5bedaff8a950b0063b1cf.fe24971839096460b051a6da5ee3a6db1224d512e1b71d4d348c1444</t>
+  </si>
+  <si>
+    <t>dNIGTH.v2</t>
+  </si>
+  <si>
+    <t>dtoken</t>
   </si>
 </sst>
 </file>
@@ -165,8 +175,8 @@
   <numFmts count="4">
     <numFmt numFmtId="176" formatCode="_-* #,##0\ &quot;₫&quot;_-;\-* #,##0\ &quot;₫&quot;_-;_-* &quot;-&quot;\ &quot;₫&quot;_-;_-@_-"/>
     <numFmt numFmtId="177" formatCode="_-* #,##0.00\ &quot;₫&quot;_-;\-* #,##0.00\ &quot;₫&quot;_-;_-* &quot;-&quot;??\ &quot;₫&quot;_-;_-@_-"/>
-    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="179" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="21">
     <font>
@@ -174,6 +184,113 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -191,47 +308,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -245,88 +331,12 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color rgb="FF9C6500"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="33">
     <fill>
@@ -337,187 +347,187 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="5" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -531,41 +541,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top/>
       <bottom style="medium">
         <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -581,17 +561,6 @@
       </top>
       <bottom style="double">
         <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -620,6 +589,21 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top/>
@@ -628,151 +612,177 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="23" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1308,7 +1318,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:H55"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75" outlineLevelCol="7"/>
   <cols>
     <col min="4" max="4" width="79.5" customWidth="1"/>
@@ -2590,35 +2600,44 @@
         <v>100000000</v>
       </c>
     </row>
-    <row r="50" spans="2:5">
-      <c r="B50" t="s">
-        <v>2</v>
-      </c>
+    <row r="50" spans="3:8">
       <c r="C50" t="s">
         <v>3</v>
       </c>
       <c r="D50" t="s">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="E50" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="51" spans="2:5">
+        <v>46</v>
+      </c>
+      <c r="H50">
+        <v>100000000</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
+      <c r="A51" t="s">
+        <v>40</v>
+      </c>
       <c r="B51" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="C51" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="D51" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E51" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="52" spans="2:5">
+        <v>29</v>
+      </c>
+      <c r="H51">
+        <v>100000000</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
+      <c r="A52" t="s">
+        <v>41</v>
+      </c>
       <c r="B52" t="s">
         <v>4</v>
       </c>
@@ -2631,37 +2650,229 @@
       <c r="E52" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="53" spans="2:5">
+      <c r="H52">
+        <v>100000000</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
+      <c r="A53" t="s">
+        <v>42</v>
+      </c>
       <c r="B53" t="s">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="C53" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="D53" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="E53" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="54" spans="3:5">
+        <v>21</v>
+      </c>
+      <c r="H53">
+        <v>100000000</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8">
+      <c r="A54" t="s">
+        <v>43</v>
+      </c>
+      <c r="B54" t="s">
+        <v>30</v>
+      </c>
       <c r="C54" t="s">
+        <v>31</v>
+      </c>
+      <c r="D54" t="s">
+        <v>47</v>
+      </c>
+      <c r="E54" t="s">
+        <v>48</v>
+      </c>
+      <c r="H54">
+        <v>100000000</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8">
+      <c r="A55" t="s">
+        <v>44</v>
+      </c>
+      <c r="C55" t="s">
         <v>3</v>
       </c>
-      <c r="D54" t="s">
-        <v>45</v>
-      </c>
-      <c r="E54" t="s">
-        <v>46</v>
+      <c r="D55" t="s">
+        <v>18</v>
+      </c>
+      <c r="E55" t="s">
+        <v>19</v>
+      </c>
+      <c r="H55">
+        <v>100000000</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A1:G49" numberStoredAsText="1"/>
+    <ignoredError sqref="A11:G49;E10:G10;A10:C10;A1:G9" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75" outlineLevelRow="5"/>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" t="str">
+        <f>"d"&amp;C2</f>
+        <v>dUSDM</v>
+      </c>
+      <c r="F2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I2" t="str">
+        <f>IF(D2=F2,"OK","False")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" t="str">
+        <f>"d"&amp;C3</f>
+        <v>dBTC</v>
+      </c>
+      <c r="F3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" t="str">
+        <f>IF(D3=F3,"OK","False")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" t="str">
+        <f>"d"&amp;C4</f>
+        <v>dUSDA</v>
+      </c>
+      <c r="F4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I4" t="str">
+        <f>IF(D4=F4,"OK","False")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" t="str">
+        <f>"d"&amp;C5</f>
+        <v>dNIGHT</v>
+      </c>
+      <c r="I5" t="str">
+        <f>IF(D5=F5,"OK","False")</f>
+        <v>False</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" t="str">
+        <f>"d"&amp;C6</f>
+        <v>dADA</v>
+      </c>
+      <c r="F6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I6" t="str">
+        <f>IF(D6=F6,"OK","False")</f>
+        <v>OK</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>